<commit_message>
tilføje værdier fra Vejdim til AKK's BG Designmanual + mindre rettelser til app'en
</commit_message>
<xml_diff>
--- a/Dokumenter og data/datablade og designmanualer/BG designmanual input til program AKK_rev 2026 DST.xlsx
+++ b/Dokumenter og data/datablade og designmanualer/BG designmanual input til program AKK_rev 2026 DST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byggrosas.sharepoint.com/sites/Byg/Shared Documents/General/Personlige mapper/BDK/Dan Strand/Beregningsværktøj/datablade og designmanualer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\geonet_beregning\Dokumenter og data\datablade og designmanualer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="257" documentId="13_ncr:1_{5DEB2B14-722A-4740-8D49-9704A1B3F39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76D8512F-EE9D-455B-9AEF-2CF4D0F40A24}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A4C94D-708B-4434-91A8-0862860FB91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="151">
   <si>
     <t>Tensar Pave</t>
   </si>
@@ -468,6 +468,30 @@
   <si>
     <t>Bundgrus 0-8</t>
   </si>
+  <si>
+    <t>reduktionsfaktor</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>T3</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>T6</t>
+  </si>
+  <si>
+    <t>T7</t>
+  </si>
 </sst>
 </file>
 
@@ -511,7 +535,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -545,6 +569,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -659,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -690,6 +720,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -11785,7 +11816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB44"/>
+  <dimension ref="A1:AC48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
@@ -12106,7 +12137,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>6</v>
       </c>
@@ -12127,10 +12158,10 @@
       </c>
       <c r="Q17" s="1"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q18" s="1"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>30</v>
       </c>
@@ -12173,7 +12204,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>6</v>
       </c>
@@ -12194,10 +12225,10 @@
       </c>
       <c r="Q20" s="1"/>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q21" s="1"/>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>40</v>
       </c>
@@ -12236,7 +12267,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>6</v>
       </c>
@@ -12257,7 +12288,7 @@
       </c>
       <c r="Q23" s="1"/>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>7</v>
       </c>
@@ -12267,8 +12298,29 @@
       <c r="R25" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="W25" t="s">
+        <v>144</v>
+      </c>
+      <c r="X25" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>149</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -12345,12 +12397,12 @@
         <v>150</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>5</v>
       </c>
@@ -12424,7 +12476,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>6</v>
       </c>
@@ -12443,12 +12495,42 @@
       <c r="G29">
         <v>1295</v>
       </c>
+      <c r="J29" s="30">
+        <f>W29*$N$48</f>
+        <v>301</v>
+      </c>
+      <c r="L29" s="30">
+        <f>Y29*$N$48</f>
+        <v>644</v>
+      </c>
+      <c r="N29" s="30">
+        <f>AA29*$N$48</f>
+        <v>826</v>
+      </c>
       <c r="Q29" s="1"/>
-    </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="W29" s="30">
+        <v>430</v>
+      </c>
+      <c r="X29" s="30">
+        <v>840</v>
+      </c>
+      <c r="Y29" s="30">
+        <v>920</v>
+      </c>
+      <c r="Z29" s="30">
+        <v>1070</v>
+      </c>
+      <c r="AA29" s="30">
+        <v>1180</v>
+      </c>
+      <c r="AB29" s="30">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q30" s="1"/>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>10</v>
       </c>
@@ -12522,7 +12604,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>6</v>
       </c>
@@ -12541,7 +12623,37 @@
       <c r="G32">
         <v>1005</v>
       </c>
+      <c r="J32" s="30">
+        <f>W32*$N$48</f>
+        <v>237.99999999999997</v>
+      </c>
+      <c r="L32" s="30">
+        <f>Y32*$N$48</f>
+        <v>546</v>
+      </c>
+      <c r="N32" s="30">
+        <f>AA32*$N$48</f>
+        <v>700</v>
+      </c>
       <c r="Q32" s="1"/>
+      <c r="W32" s="30">
+        <v>340</v>
+      </c>
+      <c r="X32" s="30">
+        <v>700</v>
+      </c>
+      <c r="Y32" s="30">
+        <v>780</v>
+      </c>
+      <c r="Z32" s="30">
+        <v>890</v>
+      </c>
+      <c r="AA32" s="30">
+        <v>1000</v>
+      </c>
+      <c r="AB32" s="30">
+        <v>1050</v>
+      </c>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q33" s="1"/>
@@ -12639,7 +12751,37 @@
       <c r="G35">
         <v>765</v>
       </c>
+      <c r="J35" s="30">
+        <f>W35*$N$48</f>
+        <v>210</v>
+      </c>
+      <c r="L35" s="30">
+        <f>Y35*$N$48</f>
+        <v>475.99999999999994</v>
+      </c>
+      <c r="N35" s="30">
+        <f>AA35*$N$48</f>
+        <v>616</v>
+      </c>
       <c r="Q35" s="1"/>
+      <c r="W35" s="30">
+        <v>300</v>
+      </c>
+      <c r="X35" s="30">
+        <v>620</v>
+      </c>
+      <c r="Y35" s="30">
+        <v>680</v>
+      </c>
+      <c r="Z35" s="30">
+        <v>790</v>
+      </c>
+      <c r="AA35" s="30">
+        <v>880</v>
+      </c>
+      <c r="AB35" s="30">
+        <v>930</v>
+      </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q36" s="1"/>
@@ -12737,7 +12879,37 @@
       <c r="G38">
         <v>620</v>
       </c>
+      <c r="J38" s="30">
+        <f>W38*$N$48</f>
+        <v>147</v>
+      </c>
+      <c r="L38" s="30">
+        <f>Y38*$N$48</f>
+        <v>434</v>
+      </c>
+      <c r="N38" s="30">
+        <f>AA38*$N$48</f>
+        <v>560</v>
+      </c>
       <c r="Q38" s="1"/>
+      <c r="W38" s="30">
+        <v>210</v>
+      </c>
+      <c r="X38" s="30">
+        <v>560</v>
+      </c>
+      <c r="Y38" s="30">
+        <v>620</v>
+      </c>
+      <c r="Z38" s="30">
+        <v>720</v>
+      </c>
+      <c r="AA38" s="30">
+        <v>800</v>
+      </c>
+      <c r="AB38" s="30">
+        <v>840</v>
+      </c>
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q39" s="1"/>
@@ -12832,7 +13004,34 @@
       <c r="G41">
         <v>450</v>
       </c>
+      <c r="J41" s="30"/>
+      <c r="L41" s="30">
+        <f>Y41*$N$48</f>
+        <v>371</v>
+      </c>
+      <c r="N41" s="30">
+        <f>AA41*$N$48</f>
+        <v>475.99999999999994</v>
+      </c>
       <c r="Q41" s="1"/>
+      <c r="W41" s="30">
+        <v>170</v>
+      </c>
+      <c r="X41" s="30">
+        <v>480</v>
+      </c>
+      <c r="Y41" s="30">
+        <v>530</v>
+      </c>
+      <c r="Z41" s="30">
+        <v>610</v>
+      </c>
+      <c r="AA41" s="30">
+        <v>680</v>
+      </c>
+      <c r="AB41" s="30">
+        <v>710</v>
+      </c>
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q42" s="1"/>
@@ -12915,7 +13114,42 @@
       <c r="G44">
         <v>345</v>
       </c>
+      <c r="J44" s="30"/>
+      <c r="L44" s="30">
+        <f>Y44*$N$48</f>
+        <v>322</v>
+      </c>
+      <c r="N44" s="30">
+        <f>AA44*$N$48</f>
+        <v>413</v>
+      </c>
       <c r="Q44" s="1"/>
+      <c r="W44" s="30">
+        <v>140</v>
+      </c>
+      <c r="X44" s="30">
+        <v>410</v>
+      </c>
+      <c r="Y44" s="30">
+        <v>460</v>
+      </c>
+      <c r="Z44" s="30">
+        <v>530</v>
+      </c>
+      <c r="AA44" s="30">
+        <v>590</v>
+      </c>
+      <c r="AB44" s="30">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="L48" t="s">
+        <v>143</v>
+      </c>
+      <c r="N48">
+        <v>0.7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17464,17 +17698,17 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -17486,17 +17720,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="41c9fafd-c058-44f8-b2ce-53cd3afba157" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c9f7625-f508-4699-980b-15a788d55c32">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -17505,7 +17728,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A8CC43999E69B146B21FD7037336070D" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="da949df7407854784e825555ef0470b6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3c9f7625-f508-4699-980b-15a788d55c32" xmlns:ns3="41c9fafd-c058-44f8-b2ce-53cd3afba157" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="15818a7baaa05f324ff0ec0f28430cf1" ns2:_="" ns3:_="">
     <xsd:import namespace="3c9f7625-f508-4699-980b-15a788d55c32"/>
@@ -17766,18 +17989,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F24CF1C-E15F-4170-99B6-AB935727F795}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="41c9fafd-c058-44f8-b2ce-53cd3afba157"/>
-    <ds:schemaRef ds:uri="3c9f7625-f508-4699-980b-15a788d55c32"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="41c9fafd-c058-44f8-b2ce-53cd3afba157" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c9f7625-f508-4699-980b-15a788d55c32">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4A9A146-E1D4-411F-BBA2-056A85056DA8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -17785,7 +18008,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{118099E9-5674-4C43-BF01-17622689F55A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17802,4 +18025,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F24CF1C-E15F-4170-99B6-AB935727F795}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="41c9fafd-c058-44f8-b2ce-53cd3afba157"/>
+    <ds:schemaRef ds:uri="3c9f7625-f508-4699-980b-15a788d55c32"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ret diverse tekster rundt om i appen og hvornår advarsler udløses. Ret at der indsættes standard teksten i rapporten, hvis man sletter et af de foruddefinerede tekstfelter
</commit_message>
<xml_diff>
--- a/Dokumenter og data/datablade og designmanualer/BG designmanual input til program AKK_rev 2026 DST.xlsx
+++ b/Dokumenter og data/datablade og designmanualer/BG designmanual input til program AKK_rev 2026 DST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\geonet_beregning\Dokumenter og data\datablade og designmanualer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A4C94D-708B-4434-91A8-0862860FB91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBBDB4A-D2E3-4DA3-BFFC-80CF7C4F3214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,10 @@
     <sheet name="Diagrammer" sheetId="6" r:id="rId3"/>
     <sheet name="Ark3" sheetId="3" r:id="rId4"/>
     <sheet name="Forsøgsbeskrivelse" sheetId="4" r:id="rId5"/>
+    <sheet name="VejDim" sheetId="7" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="157">
   <si>
     <t>Tensar Pave</t>
   </si>
@@ -490,14 +491,33 @@
     <t>T6</t>
   </si>
   <si>
-    <t>T7</t>
+    <t>(eksempel herunder fra T4)</t>
+  </si>
+  <si>
+    <t>Indtastning i gule felter ud fra vejdims dimensionering, almindelig bundsikring og stabilgrus</t>
+  </si>
+  <si>
+    <t>(Ved 30% reduktion er faktoren 0,7)</t>
+  </si>
+  <si>
+    <t>T7/NÆ10 data fra vejdim</t>
+  </si>
+  <si>
+    <t>Sammenhængen er vejledende, idet Byggros' belastningsklasser er defineret ud fra tilladt akseltryk og anvendelsesområde, mens de danske trafikklasser T0-T7 er defineret ud fra akkumulativ trafikbelastning udtrykt ved antal tunge køretøjer eller ækvivalente 10-tons aksler (NÆ10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Klasse
+Eu</t>
+  </si>
+  <si>
+    <t>Nye tabeller med opdaterede tal fra VejDim</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -534,8 +554,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -578,8 +613,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -685,11 +726,148 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalDown="1">
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal style="thin">
+        <color auto="1"/>
+      </diagonal>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -721,9 +899,54 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10631,6 +10854,215 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>44823</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>23888</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>89647</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Billede 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3D7C8CD-6F4F-872B-10E6-DCA1C32AB038}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14847794" y="1187823"/>
+          <a:ext cx="6108682" cy="3092824"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>493060</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>106456</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>89647</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>78441</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="Lige pilforbindelse 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87C473B4-CEA7-93B1-B38F-1DCCAB4B15E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="6" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="14164236" y="3535456"/>
+          <a:ext cx="4437529" cy="1876985"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="34925">
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>89647</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>33617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>56030</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>179294</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Ellipse 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8240BDED-6718-CF1B-BB20-C14E4E311466}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18601765" y="3272117"/>
+          <a:ext cx="571500" cy="526677"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="da-DK" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>33618</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>51156</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>415817</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>60290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Billede 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A4E994B-2541-7240-0338-E33409CEDD21}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17335500" y="5385156"/>
+          <a:ext cx="7038493" cy="3438134"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -11252,7 +11684,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -11326,6 +11758,1733 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>183505</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Billede 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AF64921-6926-7920-F138-A106392CC4DA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705601" y="1524001"/>
+          <a:ext cx="5669904" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>89</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>99</xdr:col>
+      <xdr:colOff>24130</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Billede 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B4EC354-F4A2-4902-A9BB-97BDB80D3585}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="54254400" y="952500"/>
+          <a:ext cx="6120130" cy="8280400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>99</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>109</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>113211</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Billede 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09EC7D62-DD5A-493E-A2B4-0D50F68AF89F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="60350400" y="1123950"/>
+          <a:ext cx="6143625" cy="3370761"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>184338</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Billede 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4F69A13-BC49-90A7-B288-09F2151B03BD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705600" y="4381500"/>
+          <a:ext cx="5670738" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>180173</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Billede 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CBC2DB1-A0C6-671B-BFE0-B3B08976E6BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705600" y="7239000"/>
+          <a:ext cx="5666573" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>180392</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Billede 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFA493D7-DE56-57FA-685D-E6170ADCB7A7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705600" y="10134601"/>
+          <a:ext cx="5715000" cy="2809290"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>253881</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Billede 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99172AA0-EBF9-E2DC-CF6E-3D109EABA5F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705601" y="12954001"/>
+          <a:ext cx="5740280" cy="2819400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>262705</xdr:colOff>
+      <xdr:row>109</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Billede 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B55A311-B878-88CD-EC83-A6F263B8972F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6705600" y="15811501"/>
+          <a:ext cx="5749105" cy="2819400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>457201</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>571499</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>141039</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Billede 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72F91C51-585C-D369-7B36-300A4B268270}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13258801" y="1600200"/>
+          <a:ext cx="5600699" cy="2731839"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>457201</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>581306</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Billede 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DC4E0484-D899-B246-14F3-39EC5D65A2D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13258801" y="4495801"/>
+          <a:ext cx="5610506" cy="2743199"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>600713</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>38099</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Billede 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A390DD90-8748-C2F7-1BEF-8FCAD4BA3827}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411201" y="7429500"/>
+          <a:ext cx="5477512" cy="2705100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>506610</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>114302</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Billede 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D674111E-6E33-B7F7-B0D1-207BD74403FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13373100" y="10401301"/>
+          <a:ext cx="5421511" cy="2667000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>381001</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>100065</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Billede 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74590263-7513-9E20-67CC-79C49B9DDFE2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411201" y="13144501"/>
+          <a:ext cx="5257800" cy="2576564"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>33695</xdr:colOff>
+      <xdr:row>109</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Billede 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BD4BDAE-5252-7527-A1DB-94CBEC8CD10A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411200" y="15811501"/>
+          <a:ext cx="5520094" cy="2705100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>38101</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>323075</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Billede 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1577634F-499D-33B1-B051-37DD54CBCFA6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19545301" y="1714500"/>
+          <a:ext cx="5771374" cy="2819400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>176309</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Billede 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73BB308C-E2AC-0CC5-B642-72E1766D667F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19507200" y="4762501"/>
+          <a:ext cx="5662709" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>189722</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Billede 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE3CD651-1D58-828D-E254-EBB8BB9CD78F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19507200" y="7620000"/>
+          <a:ext cx="5676122" cy="2781300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>190501</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>108179</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Billede 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2A3CAA9-1599-CCB1-875D-2C44E6A7707D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19507201" y="10668000"/>
+          <a:ext cx="5676900" cy="2775180"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>114301</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>304801</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>110409</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="25" name="Billede 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E93BE90B-980F-B330-B125-532DC58A0A6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19621501" y="13525500"/>
+          <a:ext cx="5676900" cy="2777408"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>604325</xdr:colOff>
+      <xdr:row>110</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Billede 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5BB6E059-A895-BF12-30AE-316CE78A0EA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19507200" y="16383000"/>
+          <a:ext cx="4871526" cy="2400300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>50</xdr:col>
+      <xdr:colOff>234909</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Billede 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A5015E7-071D-6B08-EEF7-5267557E860C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603201" y="1714501"/>
+          <a:ext cx="5111708" cy="2514599"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>50</xdr:col>
+      <xdr:colOff>103193</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Billede 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF304CC1-A86D-7BEF-DB76-AA06C7AA0D2D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603201" y="4762500"/>
+          <a:ext cx="4979992" cy="2438400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>475862</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>38099</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Billede 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D895E6F8-00CB-7348-DCCD-D08FFA554495}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603200" y="7810500"/>
+          <a:ext cx="4743061" cy="2324100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>476010</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Billede 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B1F3765-7C66-C465-133D-57DB80CDF71C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603200" y="10820400"/>
+          <a:ext cx="4743209" cy="2324100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>564913</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Billede 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB25D967-F168-69F0-022D-F2863622CE4C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603201" y="13716000"/>
+          <a:ext cx="4832111" cy="2362200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>397962</xdr:colOff>
+      <xdr:row>111</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Billede 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D36CA84F-914C-8EFC-F159-F3EF8406C361}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25603201" y="16573500"/>
+          <a:ext cx="4665160" cy="2286000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>410051</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Billede 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E92277A-4FFF-EBC2-AC07-FA978B84A328}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699200" y="1714501"/>
+          <a:ext cx="5286851" cy="2590800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>304147</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="34" name="Billede 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED74D8EF-92EB-D9DD-75A7-004C316A14F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699200" y="4762500"/>
+          <a:ext cx="5180947" cy="2552700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>246404</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>38099</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Billede 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2549A88D-F858-0E8D-1CB7-037421AAB6AD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699201" y="7810500"/>
+          <a:ext cx="5123203" cy="2514600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>10197</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Billede 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA381407-7DE9-F427-D4D7-2BE6E9838501}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699201" y="10858501"/>
+          <a:ext cx="4886996" cy="2400300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>36844</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="37" name="Billede 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44F36CAB-5EF5-3D80-5328-AA61F2C7033E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699200" y="13716000"/>
+          <a:ext cx="4913644" cy="2400300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>266699</xdr:colOff>
+      <xdr:row>110</xdr:row>
+      <xdr:rowOff>131437</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="Billede 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0226A4B2-B1A4-B073-0F39-E35C6A23279A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31699201" y="16573501"/>
+          <a:ext cx="4533899" cy="2226935"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>76201</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>69</xdr:col>
+      <xdr:colOff>521416</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="39" name="Billede 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F8F6464-0601-0CF4-CCCD-1AC8FB6BD66A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37452300" y="1790701"/>
+          <a:ext cx="5131515" cy="2514600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>266701</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>152401</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>170382</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="Billede 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8A9E008-2720-14FF-6994-7352495DCCA9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37452301" y="4572000"/>
+          <a:ext cx="5372100" cy="2646883"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>304801</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>163022</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Billede 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8619277A-1819-8086-BE5A-7EEA41006352}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37490401" y="7658100"/>
+          <a:ext cx="5295899" cy="2601423"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>304801</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>36007</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Billede 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B33FABC9-7C35-B289-358F-6ACE818F297D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37490401" y="10668000"/>
+          <a:ext cx="5217606" cy="2552700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>73307</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="43" name="Billede 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25FE5A32-40AD-F2CE-6262-155C8C337F03}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37566600" y="13716000"/>
+          <a:ext cx="5219700" cy="2549807"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>342901</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>70</xdr:col>
+      <xdr:colOff>152401</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>167070</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="44" name="Billede 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98F0F644-5F27-51EC-FAA4-D35A0437560C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="37528501" y="16611600"/>
+          <a:ext cx="5295900" cy="2605469"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>101</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>111</xdr:col>
+      <xdr:colOff>102200</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="45" name="Billede 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5340A34F-8C6A-4479-BE8B-289F91E36BCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="61569600" y="5715000"/>
+          <a:ext cx="6198199" cy="2171700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -11505,6 +13664,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11794,7 +13957,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="10">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="11">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -11816,7 +13979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC48"/>
+  <dimension ref="A1:AF67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
@@ -11825,12 +13988,12 @@
     <col min="16" max="16" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -11838,7 +14001,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
         <v>10</v>
       </c>
@@ -11852,7 +14015,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -11863,7 +14026,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -11903,13 +14066,19 @@
       <c r="V5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="AB5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="AB6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -11950,7 +14119,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -11971,10 +14140,10 @@
       </c>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -12012,7 +14181,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>6</v>
       </c>
@@ -12033,10 +14202,10 @@
       </c>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>15</v>
       </c>
@@ -12074,7 +14243,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>6</v>
       </c>
@@ -12095,10 +14264,10 @@
       </c>
       <c r="Q14" s="1"/>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="Q15" s="1"/>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>20</v>
       </c>
@@ -12137,7 +14306,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>6</v>
       </c>
@@ -12158,10 +14327,10 @@
       </c>
       <c r="Q17" s="1"/>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="Q18" s="1"/>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>30</v>
       </c>
@@ -12204,7 +14373,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>6</v>
       </c>
@@ -12225,10 +14394,10 @@
       </c>
       <c r="Q20" s="1"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="Q21" s="1"/>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>40</v>
       </c>
@@ -12267,7 +14436,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>6</v>
       </c>
@@ -12288,7 +14457,7 @@
       </c>
       <c r="Q23" s="1"/>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>7</v>
       </c>
@@ -12298,29 +14467,27 @@
       <c r="R25" t="s">
         <v>8</v>
       </c>
-      <c r="W25" t="s">
+      <c r="W25" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="X25" t="s">
+      <c r="X25" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="Y25" t="s">
+      <c r="Y25" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="Z25" t="s">
+      <c r="Z25" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="AA25" t="s">
+      <c r="AA25" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="AB25" t="s">
+      <c r="AB25" s="31" t="s">
         <v>149</v>
       </c>
-      <c r="AC25" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AC25" s="31"/>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>4</v>
       </c>
@@ -12397,12 +14564,12 @@
         <v>150</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>5</v>
       </c>
@@ -12475,8 +14642,11 @@
       <c r="AB28">
         <v>1400</v>
       </c>
-    </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AF28" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>6</v>
       </c>
@@ -12496,16 +14666,28 @@
         <v>1295</v>
       </c>
       <c r="J29" s="30">
-        <f>W29*$N$48</f>
+        <f>W29*$L$46</f>
         <v>301</v>
       </c>
+      <c r="K29" s="30">
+        <f>X29*$L$46</f>
+        <v>588</v>
+      </c>
       <c r="L29" s="30">
-        <f>Y29*$N$48</f>
+        <f>Y29*$L$46</f>
         <v>644</v>
       </c>
+      <c r="M29" s="30">
+        <f>Z29*$L$46</f>
+        <v>749</v>
+      </c>
       <c r="N29" s="30">
-        <f>AA29*$N$48</f>
+        <f>AA29*$L$46</f>
         <v>826</v>
+      </c>
+      <c r="O29" s="30">
+        <f>AB29*$L$46</f>
+        <v>875</v>
       </c>
       <c r="Q29" s="1"/>
       <c r="W29" s="30">
@@ -12526,11 +14708,12 @@
       <c r="AB29" s="30">
         <v>1250</v>
       </c>
-    </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="AC29" s="30"/>
+    </row>
+    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="Q30" s="1"/>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>10</v>
       </c>
@@ -12604,7 +14787,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>6</v>
       </c>
@@ -12624,16 +14807,28 @@
         <v>1005</v>
       </c>
       <c r="J32" s="30">
-        <f>W32*$N$48</f>
+        <f>W32*$L$46</f>
         <v>237.99999999999997</v>
       </c>
+      <c r="K32" s="30">
+        <f>X32*$L$46</f>
+        <v>489.99999999999994</v>
+      </c>
       <c r="L32" s="30">
-        <f>Y32*$N$48</f>
+        <f>Y32*$L$46</f>
         <v>546</v>
       </c>
+      <c r="M32" s="30">
+        <f>Z32*$L$46</f>
+        <v>623</v>
+      </c>
       <c r="N32" s="30">
-        <f>AA32*$N$48</f>
+        <f>AA32*$L$46</f>
         <v>700</v>
+      </c>
+      <c r="O32" s="30">
+        <f>AB32*$L$46</f>
+        <v>735</v>
       </c>
       <c r="Q32" s="1"/>
       <c r="W32" s="30">
@@ -12654,11 +14849,12 @@
       <c r="AB32" s="30">
         <v>1050</v>
       </c>
-    </row>
-    <row r="33" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC32" s="30"/>
+    </row>
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>15</v>
       </c>
@@ -12732,7 +14928,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="35" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>6</v>
       </c>
@@ -12752,16 +14948,28 @@
         <v>765</v>
       </c>
       <c r="J35" s="30">
-        <f>W35*$N$48</f>
+        <f>W35*$L$46</f>
         <v>210</v>
       </c>
+      <c r="K35" s="30">
+        <f>X35*$L$46</f>
+        <v>434</v>
+      </c>
       <c r="L35" s="30">
-        <f>Y35*$N$48</f>
+        <f>Y35*$L$46</f>
         <v>475.99999999999994</v>
       </c>
+      <c r="M35" s="30">
+        <f>Z35*$L$46</f>
+        <v>553</v>
+      </c>
       <c r="N35" s="30">
-        <f>AA35*$N$48</f>
+        <f>AA35*$L$46</f>
         <v>616</v>
+      </c>
+      <c r="O35" s="30">
+        <f>AB35*$L$46</f>
+        <v>651</v>
       </c>
       <c r="Q35" s="1"/>
       <c r="W35" s="30">
@@ -12782,11 +14990,12 @@
       <c r="AB35" s="30">
         <v>930</v>
       </c>
-    </row>
-    <row r="36" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC35" s="30"/>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q36" s="1"/>
     </row>
-    <row r="37" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>20</v>
       </c>
@@ -12860,7 +15069,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="38" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>6</v>
       </c>
@@ -12880,16 +15089,28 @@
         <v>620</v>
       </c>
       <c r="J38" s="30">
-        <f>W38*$N$48</f>
+        <f>W38*$L$46</f>
         <v>147</v>
       </c>
+      <c r="K38" s="30">
+        <f>X38*$L$46</f>
+        <v>392</v>
+      </c>
       <c r="L38" s="30">
-        <f>Y38*$N$48</f>
+        <f>Y38*$L$46</f>
         <v>434</v>
       </c>
+      <c r="M38" s="30">
+        <f>Z38*$L$46</f>
+        <v>503.99999999999994</v>
+      </c>
       <c r="N38" s="30">
-        <f>AA38*$N$48</f>
+        <f>AA38*$L$46</f>
         <v>560</v>
+      </c>
+      <c r="O38" s="30">
+        <f>AB38*$L$46</f>
+        <v>588</v>
       </c>
       <c r="Q38" s="1"/>
       <c r="W38" s="30">
@@ -12910,11 +15131,12 @@
       <c r="AB38" s="30">
         <v>840</v>
       </c>
-    </row>
-    <row r="39" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC38" s="30"/>
+    </row>
+    <row r="39" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q39" s="1"/>
     </row>
-    <row r="40" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>30</v>
       </c>
@@ -12985,7 +15207,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>6</v>
       </c>
@@ -13006,12 +15228,16 @@
       </c>
       <c r="J41" s="30"/>
       <c r="L41" s="30">
-        <f>Y41*$N$48</f>
+        <f>Y41*$L$46</f>
         <v>371</v>
       </c>
       <c r="N41" s="30">
-        <f>AA41*$N$48</f>
+        <f>AA41*$L$46</f>
         <v>475.99999999999994</v>
+      </c>
+      <c r="O41" s="30">
+        <f>AB41*$L$46</f>
+        <v>496.99999999999994</v>
       </c>
       <c r="Q41" s="1"/>
       <c r="W41" s="30">
@@ -13032,11 +15258,12 @@
       <c r="AB41" s="30">
         <v>710</v>
       </c>
-    </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC41" s="30"/>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="Q42" s="1"/>
     </row>
-    <row r="43" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>40</v>
       </c>
@@ -13095,7 +15322,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="44" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>6</v>
       </c>
@@ -13116,12 +15343,16 @@
       </c>
       <c r="J44" s="30"/>
       <c r="L44" s="30">
-        <f>Y44*$N$48</f>
+        <f>Y44*$L$46</f>
         <v>322</v>
       </c>
       <c r="N44" s="30">
-        <f>AA44*$N$48</f>
+        <f>AA44*$L$46</f>
         <v>413</v>
+      </c>
+      <c r="O44" s="30">
+        <f>AB44*$L$46</f>
+        <v>434</v>
       </c>
       <c r="Q44" s="1"/>
       <c r="W44" s="30">
@@ -13142,18 +15373,588 @@
       <c r="AB44" s="30">
         <v>620</v>
       </c>
-    </row>
-    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="L48" t="s">
+      <c r="AC44" s="30"/>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="J46" t="s">
         <v>143</v>
       </c>
-      <c r="N48">
+      <c r="L46">
         <v>0.7</v>
+      </c>
+      <c r="M46" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="47" spans="1:29" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="48" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="W48" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="X48" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y48" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z48" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA48" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB48" s="31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="49" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="H49" t="s">
+        <v>4</v>
+      </c>
+      <c r="J49">
+        <v>30</v>
+      </c>
+      <c r="K49">
+        <v>45</v>
+      </c>
+      <c r="L49">
+        <v>60</v>
+      </c>
+      <c r="M49">
+        <v>80</v>
+      </c>
+      <c r="N49">
+        <v>120</v>
+      </c>
+      <c r="O49">
+        <v>150</v>
+      </c>
+      <c r="V49" t="s">
+        <v>4</v>
+      </c>
+      <c r="W49">
+        <v>30</v>
+      </c>
+      <c r="X49">
+        <v>45</v>
+      </c>
+      <c r="Y49">
+        <v>60</v>
+      </c>
+      <c r="Z49">
+        <v>80</v>
+      </c>
+      <c r="AA49">
+        <v>120</v>
+      </c>
+      <c r="AB49">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="50" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
+        <v>1</v>
+      </c>
+      <c r="U50" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G51">
+        <v>5</v>
+      </c>
+      <c r="J51">
+        <v>600</v>
+      </c>
+      <c r="K51">
+        <v>680</v>
+      </c>
+      <c r="L51">
+        <v>800</v>
+      </c>
+      <c r="M51">
+        <v>900</v>
+      </c>
+      <c r="N51">
+        <v>950</v>
+      </c>
+      <c r="O51">
+        <v>1000</v>
+      </c>
+      <c r="U51">
+        <v>5</v>
+      </c>
+      <c r="W51">
+        <v>900</v>
+      </c>
+      <c r="X51">
+        <v>1000</v>
+      </c>
+      <c r="Y51">
+        <v>1110</v>
+      </c>
+      <c r="Z51">
+        <v>1200</v>
+      </c>
+      <c r="AA51">
+        <v>1300</v>
+      </c>
+      <c r="AB51">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="52" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J52" s="30">
+        <f>W52*$L$46</f>
+        <v>329</v>
+      </c>
+      <c r="K52" s="30">
+        <f>X52*$L$46</f>
+        <v>651</v>
+      </c>
+      <c r="L52" s="30">
+        <f>Y52*$L$46</f>
+        <v>714</v>
+      </c>
+      <c r="M52" s="30">
+        <f>Z52*$L$46</f>
+        <v>833</v>
+      </c>
+      <c r="N52" s="30">
+        <f>AA52*$L$46</f>
+        <v>916.99999999999989</v>
+      </c>
+      <c r="O52" s="30">
+        <f>AB52*$L$46</f>
+        <v>965.99999999999989</v>
+      </c>
+      <c r="W52" s="47">
+        <v>470</v>
+      </c>
+      <c r="X52" s="47">
+        <v>930</v>
+      </c>
+      <c r="Y52" s="47">
+        <v>1020</v>
+      </c>
+      <c r="Z52" s="47">
+        <v>1190</v>
+      </c>
+      <c r="AA52" s="47">
+        <v>1310</v>
+      </c>
+      <c r="AB52" s="47">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="54" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G54">
+        <v>10</v>
+      </c>
+      <c r="J54">
+        <v>350</v>
+      </c>
+      <c r="K54">
+        <v>480</v>
+      </c>
+      <c r="L54">
+        <v>560</v>
+      </c>
+      <c r="M54">
+        <v>600</v>
+      </c>
+      <c r="N54">
+        <v>700</v>
+      </c>
+      <c r="O54">
+        <v>770</v>
+      </c>
+      <c r="U54">
+        <v>10</v>
+      </c>
+      <c r="W54">
+        <v>600</v>
+      </c>
+      <c r="X54">
+        <v>700</v>
+      </c>
+      <c r="Y54">
+        <v>800</v>
+      </c>
+      <c r="Z54">
+        <v>900</v>
+      </c>
+      <c r="AA54">
+        <v>1000</v>
+      </c>
+      <c r="AB54">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="55" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J55" s="30">
+        <f>W55*$L$46</f>
+        <v>251.99999999999997</v>
+      </c>
+      <c r="K55" s="30">
+        <f>X55*$L$46</f>
+        <v>532</v>
+      </c>
+      <c r="L55" s="30">
+        <f>Y55*$L$46</f>
+        <v>588</v>
+      </c>
+      <c r="M55" s="30">
+        <f>Z55*$L$46</f>
+        <v>672</v>
+      </c>
+      <c r="N55" s="30">
+        <f>AA55*$L$46</f>
+        <v>735</v>
+      </c>
+      <c r="O55" s="30">
+        <f>AB55*$L$46</f>
+        <v>812</v>
+      </c>
+      <c r="W55" s="47">
+        <v>360</v>
+      </c>
+      <c r="X55" s="47">
+        <v>760</v>
+      </c>
+      <c r="Y55" s="47">
+        <v>840</v>
+      </c>
+      <c r="Z55" s="47">
+        <v>960</v>
+      </c>
+      <c r="AA55" s="47">
+        <v>1050</v>
+      </c>
+      <c r="AB55" s="47">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="57" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G57">
+        <v>15</v>
+      </c>
+      <c r="J57">
+        <v>200</v>
+      </c>
+      <c r="K57">
+        <v>320</v>
+      </c>
+      <c r="L57">
+        <v>400</v>
+      </c>
+      <c r="M57">
+        <v>480</v>
+      </c>
+      <c r="N57">
+        <v>580</v>
+      </c>
+      <c r="O57">
+        <v>650</v>
+      </c>
+      <c r="U57">
+        <v>15</v>
+      </c>
+      <c r="W57">
+        <v>400</v>
+      </c>
+      <c r="X57">
+        <v>500</v>
+      </c>
+      <c r="Y57">
+        <v>600</v>
+      </c>
+      <c r="Z57">
+        <v>700</v>
+      </c>
+      <c r="AA57">
+        <v>800</v>
+      </c>
+      <c r="AB57">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="58" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J58" s="30">
+        <f>W58*$L$46</f>
+        <v>210</v>
+      </c>
+      <c r="K58" s="30">
+        <f>X58*$L$46</f>
+        <v>468.99999999999994</v>
+      </c>
+      <c r="L58" s="30">
+        <f>Y58*$L$46</f>
+        <v>503.99999999999994</v>
+      </c>
+      <c r="M58" s="30">
+        <f>Z58*$L$46</f>
+        <v>595</v>
+      </c>
+      <c r="N58" s="30">
+        <f>AA58*$L$46</f>
+        <v>637</v>
+      </c>
+      <c r="O58" s="30">
+        <f>AB58*$L$46</f>
+        <v>679</v>
+      </c>
+      <c r="W58" s="47">
+        <v>300</v>
+      </c>
+      <c r="X58" s="47">
+        <v>670</v>
+      </c>
+      <c r="Y58" s="47">
+        <v>720</v>
+      </c>
+      <c r="Z58" s="47">
+        <v>850</v>
+      </c>
+      <c r="AA58" s="47">
+        <v>910</v>
+      </c>
+      <c r="AB58" s="47">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="60" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G60">
+        <v>20</v>
+      </c>
+      <c r="J60" s="1">
+        <v>200</v>
+      </c>
+      <c r="K60">
+        <v>200</v>
+      </c>
+      <c r="L60">
+        <v>300</v>
+      </c>
+      <c r="M60">
+        <v>240</v>
+      </c>
+      <c r="N60">
+        <v>480</v>
+      </c>
+      <c r="O60">
+        <v>560</v>
+      </c>
+      <c r="U60">
+        <v>20</v>
+      </c>
+      <c r="W60">
+        <v>250</v>
+      </c>
+      <c r="X60">
+        <v>375</v>
+      </c>
+      <c r="Y60">
+        <v>500</v>
+      </c>
+      <c r="Z60">
+        <v>600</v>
+      </c>
+      <c r="AA60">
+        <v>680</v>
+      </c>
+      <c r="AB60">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="61" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J61" s="30">
+        <f>W61*$L$46</f>
+        <v>210</v>
+      </c>
+      <c r="K61" s="30">
+        <f>X61*$L$46</f>
+        <v>413</v>
+      </c>
+      <c r="L61" s="30">
+        <f>Y61*$L$46</f>
+        <v>448</v>
+      </c>
+      <c r="M61" s="30">
+        <f>Z61*$L$46</f>
+        <v>525</v>
+      </c>
+      <c r="N61" s="30">
+        <f>AA61*$L$46</f>
+        <v>630</v>
+      </c>
+      <c r="O61" s="30">
+        <f>AB61*$L$46</f>
+        <v>672</v>
+      </c>
+      <c r="W61" s="47">
+        <v>300</v>
+      </c>
+      <c r="X61" s="47">
+        <v>590</v>
+      </c>
+      <c r="Y61" s="47">
+        <v>640</v>
+      </c>
+      <c r="Z61" s="47">
+        <v>750</v>
+      </c>
+      <c r="AA61" s="47">
+        <v>900</v>
+      </c>
+      <c r="AB61" s="47">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="63" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G63">
+        <v>30</v>
+      </c>
+      <c r="K63" s="1">
+        <v>200</v>
+      </c>
+      <c r="L63" s="1">
+        <v>200</v>
+      </c>
+      <c r="M63" s="1">
+        <v>200</v>
+      </c>
+      <c r="N63" s="2">
+        <v>330</v>
+      </c>
+      <c r="O63" s="2">
+        <v>500</v>
+      </c>
+      <c r="U63">
+        <v>30</v>
+      </c>
+      <c r="W63">
+        <v>0</v>
+      </c>
+      <c r="X63">
+        <v>200</v>
+      </c>
+      <c r="Y63">
+        <v>300</v>
+      </c>
+      <c r="Z63">
+        <v>400</v>
+      </c>
+      <c r="AA63">
+        <v>490</v>
+      </c>
+      <c r="AB63">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="64" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J64" s="30"/>
+      <c r="L64" s="30">
+        <f>Y64*$L$46</f>
+        <v>364</v>
+      </c>
+      <c r="N64" s="30">
+        <f>AA64*$L$46</f>
+        <v>496.99999999999994</v>
+      </c>
+      <c r="O64" s="30">
+        <f>AB64*$L$46</f>
+        <v>539</v>
+      </c>
+      <c r="W64" s="47">
+        <v>300</v>
+      </c>
+      <c r="X64" s="47">
+        <v>490</v>
+      </c>
+      <c r="Y64" s="47">
+        <v>520</v>
+      </c>
+      <c r="Z64" s="47">
+        <v>640</v>
+      </c>
+      <c r="AA64" s="47">
+        <v>710</v>
+      </c>
+      <c r="AB64" s="47">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="66" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="G66">
+        <v>40</v>
+      </c>
+      <c r="N66" s="1">
+        <v>200</v>
+      </c>
+      <c r="O66">
+        <v>420</v>
+      </c>
+      <c r="U66">
+        <v>40</v>
+      </c>
+      <c r="X66">
+        <v>50</v>
+      </c>
+      <c r="Y66">
+        <v>150</v>
+      </c>
+      <c r="Z66">
+        <v>250</v>
+      </c>
+      <c r="AA66">
+        <v>360</v>
+      </c>
+      <c r="AB66">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="67" spans="7:28" x14ac:dyDescent="0.25">
+      <c r="J67" s="30"/>
+      <c r="L67" s="30">
+        <f>Y67*$L$46</f>
+        <v>336</v>
+      </c>
+      <c r="N67" s="30">
+        <f>AA67*$L$46</f>
+        <v>413</v>
+      </c>
+      <c r="O67" s="30">
+        <f>AB67*$L$46</f>
+        <v>448</v>
+      </c>
+      <c r="W67" s="47">
+        <v>300</v>
+      </c>
+      <c r="X67" s="47">
+        <v>490</v>
+      </c>
+      <c r="Y67" s="47">
+        <v>480</v>
+      </c>
+      <c r="Z67" s="47">
+        <v>530</v>
+      </c>
+      <c r="AA67" s="47">
+        <v>590</v>
+      </c>
+      <c r="AB67" s="47">
+        <v>640</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -17698,17 +20499,17 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -17719,16 +20520,638 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7799C8A9-EEB0-4C85-90C1-A6115AC4B383}">
+  <dimension ref="H3:CL116"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="14.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="8:90" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="8:90" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="J4" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="K4" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="L4" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="M4" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="N4" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q4" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="R4" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="S4" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="T4" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="U4" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="V4" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="W4" s="37" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="H5" s="38">
+        <v>5</v>
+      </c>
+      <c r="I5" s="35">
+        <v>470</v>
+      </c>
+      <c r="J5" s="35">
+        <v>930</v>
+      </c>
+      <c r="K5" s="35">
+        <v>1019</v>
+      </c>
+      <c r="L5" s="35">
+        <v>1190</v>
+      </c>
+      <c r="M5" s="35">
+        <v>1312</v>
+      </c>
+      <c r="N5" s="39">
+        <v>1384</v>
+      </c>
+      <c r="Q5" s="38">
+        <v>5</v>
+      </c>
+      <c r="R5" s="35">
+        <v>470</v>
+      </c>
+      <c r="S5" s="35">
+        <v>930</v>
+      </c>
+      <c r="T5" s="43">
+        <v>1020</v>
+      </c>
+      <c r="U5" s="43">
+        <v>1190</v>
+      </c>
+      <c r="V5" s="43">
+        <v>1310</v>
+      </c>
+      <c r="W5" s="44">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="6" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="H6" s="38">
+        <v>10</v>
+      </c>
+      <c r="I6" s="35">
+        <v>360</v>
+      </c>
+      <c r="J6" s="35">
+        <v>760</v>
+      </c>
+      <c r="K6" s="35">
+        <v>838</v>
+      </c>
+      <c r="L6" s="35">
+        <v>961</v>
+      </c>
+      <c r="M6" s="35">
+        <v>1047</v>
+      </c>
+      <c r="N6" s="39">
+        <v>1156</v>
+      </c>
+      <c r="Q6" s="38">
+        <v>10</v>
+      </c>
+      <c r="R6" s="35">
+        <v>360</v>
+      </c>
+      <c r="S6" s="35">
+        <v>760</v>
+      </c>
+      <c r="T6" s="43">
+        <v>840</v>
+      </c>
+      <c r="U6" s="43">
+        <v>960</v>
+      </c>
+      <c r="V6" s="43">
+        <v>1050</v>
+      </c>
+      <c r="W6" s="44">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="7" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="H7" s="38">
+        <v>15</v>
+      </c>
+      <c r="I7" s="35">
+        <v>300</v>
+      </c>
+      <c r="J7" s="35">
+        <v>670</v>
+      </c>
+      <c r="K7" s="35">
+        <v>722</v>
+      </c>
+      <c r="L7" s="35">
+        <v>846</v>
+      </c>
+      <c r="M7" s="35">
+        <v>912</v>
+      </c>
+      <c r="N7" s="39">
+        <v>973</v>
+      </c>
+      <c r="Q7" s="38">
+        <v>15</v>
+      </c>
+      <c r="R7" s="35">
+        <v>300</v>
+      </c>
+      <c r="S7" s="35">
+        <v>670</v>
+      </c>
+      <c r="T7" s="43">
+        <v>720</v>
+      </c>
+      <c r="U7" s="43">
+        <v>850</v>
+      </c>
+      <c r="V7" s="43">
+        <v>910</v>
+      </c>
+      <c r="W7" s="44">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="8" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="H8" s="38">
+        <v>20</v>
+      </c>
+      <c r="I8" s="35">
+        <v>300</v>
+      </c>
+      <c r="J8" s="35">
+        <v>590</v>
+      </c>
+      <c r="K8" s="35">
+        <v>640</v>
+      </c>
+      <c r="L8" s="35">
+        <v>749</v>
+      </c>
+      <c r="M8" s="35">
+        <v>899</v>
+      </c>
+      <c r="N8" s="39">
+        <v>956</v>
+      </c>
+      <c r="Q8" s="38">
+        <v>20</v>
+      </c>
+      <c r="R8" s="35">
+        <v>300</v>
+      </c>
+      <c r="S8" s="35">
+        <v>590</v>
+      </c>
+      <c r="T8" s="43">
+        <v>640</v>
+      </c>
+      <c r="U8" s="43">
+        <v>750</v>
+      </c>
+      <c r="V8" s="43">
+        <v>900</v>
+      </c>
+      <c r="W8" s="44">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="9" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="H9" s="38">
+        <v>30</v>
+      </c>
+      <c r="I9" s="35">
+        <v>300</v>
+      </c>
+      <c r="J9" s="35">
+        <v>490</v>
+      </c>
+      <c r="K9" s="35">
+        <v>524</v>
+      </c>
+      <c r="L9" s="35">
+        <v>638</v>
+      </c>
+      <c r="M9" s="35">
+        <v>706</v>
+      </c>
+      <c r="N9" s="39">
+        <v>766</v>
+      </c>
+      <c r="Q9" s="38">
+        <v>30</v>
+      </c>
+      <c r="R9" s="35">
+        <v>300</v>
+      </c>
+      <c r="S9" s="35">
+        <v>490</v>
+      </c>
+      <c r="T9" s="43">
+        <v>520</v>
+      </c>
+      <c r="U9" s="43">
+        <v>640</v>
+      </c>
+      <c r="V9" s="43">
+        <v>710</v>
+      </c>
+      <c r="W9" s="44">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="10" spans="8:90" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="40">
+        <v>40</v>
+      </c>
+      <c r="I10" s="41">
+        <v>300</v>
+      </c>
+      <c r="J10" s="41">
+        <v>490</v>
+      </c>
+      <c r="K10" s="41">
+        <v>478</v>
+      </c>
+      <c r="L10" s="41">
+        <v>527</v>
+      </c>
+      <c r="M10" s="41">
+        <v>593</v>
+      </c>
+      <c r="N10" s="42">
+        <v>644</v>
+      </c>
+      <c r="Q10" s="40">
+        <v>40</v>
+      </c>
+      <c r="R10" s="41">
+        <v>300</v>
+      </c>
+      <c r="S10" s="41">
+        <v>490</v>
+      </c>
+      <c r="T10" s="45">
+        <v>480</v>
+      </c>
+      <c r="U10" s="45">
+        <v>530</v>
+      </c>
+      <c r="V10" s="45">
+        <v>590</v>
+      </c>
+      <c r="W10" s="46">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="14" spans="8:90" x14ac:dyDescent="0.25">
+      <c r="CL14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="10:65" x14ac:dyDescent="0.25">
+      <c r="O17" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>145</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>146</v>
+      </c>
+      <c r="AT17" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD17" t="s">
+        <v>148</v>
+      </c>
+      <c r="BM17" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J27" s="33"/>
+    </row>
+    <row r="28" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J28" s="33"/>
+    </row>
+    <row r="29" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J29" s="33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J30" s="33"/>
+    </row>
+    <row r="31" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J31" s="33"/>
+    </row>
+    <row r="32" spans="10:65" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J32" s="33"/>
+    </row>
+    <row r="33" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J33" s="33"/>
+    </row>
+    <row r="34" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J34" s="33"/>
+    </row>
+    <row r="35" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J35" s="33"/>
+    </row>
+    <row r="36" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J36" s="33"/>
+    </row>
+    <row r="37" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J37" s="33"/>
+    </row>
+    <row r="38" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J38" s="33"/>
+    </row>
+    <row r="39" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J39" s="33"/>
+    </row>
+    <row r="40" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J40" s="33"/>
+    </row>
+    <row r="41" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J41" s="33">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J42" s="33"/>
+    </row>
+    <row r="43" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J43" s="33"/>
+    </row>
+    <row r="44" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J44" s="33"/>
+    </row>
+    <row r="45" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J45" s="33"/>
+    </row>
+    <row r="46" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J46" s="33"/>
+    </row>
+    <row r="47" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J47" s="33"/>
+    </row>
+    <row r="48" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J48" s="33"/>
+    </row>
+    <row r="49" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J49" s="33"/>
+    </row>
+    <row r="50" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J50" s="33"/>
+    </row>
+    <row r="51" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J51" s="33"/>
+    </row>
+    <row r="52" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J52" s="33"/>
+    </row>
+    <row r="53" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J53" s="33"/>
+    </row>
+    <row r="54" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J54" s="33">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J55" s="33"/>
+    </row>
+    <row r="56" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J56" s="33"/>
+    </row>
+    <row r="57" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J57" s="33"/>
+    </row>
+    <row r="58" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J58" s="33"/>
+    </row>
+    <row r="59" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J59" s="33"/>
+    </row>
+    <row r="60" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J60" s="33"/>
+    </row>
+    <row r="61" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J61" s="33"/>
+    </row>
+    <row r="62" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J62" s="33"/>
+    </row>
+    <row r="63" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J63" s="33"/>
+    </row>
+    <row r="64" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J64" s="33"/>
+    </row>
+    <row r="65" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J65" s="33"/>
+    </row>
+    <row r="66" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J66" s="33"/>
+    </row>
+    <row r="67" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J67" s="33"/>
+    </row>
+    <row r="68" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J68" s="33"/>
+    </row>
+    <row r="69" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J69" s="33"/>
+    </row>
+    <row r="70" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J70" s="33"/>
+    </row>
+    <row r="71" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J71" s="33"/>
+    </row>
+    <row r="72" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J72" s="33">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J73" s="33"/>
+    </row>
+    <row r="74" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J74" s="33"/>
+    </row>
+    <row r="75" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J75" s="33"/>
+    </row>
+    <row r="76" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J76" s="33"/>
+    </row>
+    <row r="77" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J77" s="33"/>
+    </row>
+    <row r="78" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J78" s="33"/>
+    </row>
+    <row r="79" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J79" s="33"/>
+    </row>
+    <row r="80" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J80" s="33"/>
+    </row>
+    <row r="81" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J81" s="33"/>
+    </row>
+    <row r="82" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J82" s="33"/>
+    </row>
+    <row r="83" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J83" s="33"/>
+    </row>
+    <row r="84" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J84" s="33"/>
+    </row>
+    <row r="85" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J85" s="33"/>
+    </row>
+    <row r="86" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J86" s="33"/>
+    </row>
+    <row r="87" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J87" s="33">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="88" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J88" s="33"/>
+    </row>
+    <row r="89" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J89" s="33"/>
+    </row>
+    <row r="90" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J90" s="33"/>
+    </row>
+    <row r="91" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J91" s="33"/>
+    </row>
+    <row r="92" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J92" s="33"/>
+    </row>
+    <row r="93" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J93" s="33"/>
+    </row>
+    <row r="94" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J94" s="33"/>
+    </row>
+    <row r="95" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J95" s="33"/>
+    </row>
+    <row r="96" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J96" s="33"/>
+    </row>
+    <row r="97" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J97" s="33"/>
+    </row>
+    <row r="98" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J98" s="33"/>
+    </row>
+    <row r="99" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J99" s="33"/>
+    </row>
+    <row r="100" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J100" s="33"/>
+    </row>
+    <row r="101" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J101" s="33"/>
+    </row>
+    <row r="102" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J102" s="33">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="103" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J103" s="33"/>
+    </row>
+    <row r="104" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J104" s="33"/>
+    </row>
+    <row r="105" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J105" s="33"/>
+    </row>
+    <row r="106" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J106" s="33"/>
+    </row>
+    <row r="107" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J107" s="33"/>
+    </row>
+    <row r="108" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J108" s="33"/>
+    </row>
+    <row r="109" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J109" s="33"/>
+    </row>
+    <row r="110" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J110" s="33"/>
+    </row>
+    <row r="111" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J111" s="33"/>
+    </row>
+    <row r="112" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J112" s="33"/>
+    </row>
+    <row r="113" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J113" s="33"/>
+    </row>
+    <row r="114" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J114" s="33"/>
+    </row>
+    <row r="115" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J115" s="33"/>
+    </row>
+    <row r="116" spans="10:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J116" s="33"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A8CC43999E69B146B21FD7037336070D" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="da949df7407854784e825555ef0470b6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3c9f7625-f508-4699-980b-15a788d55c32" xmlns:ns3="41c9fafd-c058-44f8-b2ce-53cd3afba157" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="15818a7baaa05f324ff0ec0f28430cf1" ns2:_="" ns3:_="">
     <xsd:import namespace="3c9f7625-f508-4699-980b-15a788d55c32"/>
@@ -17989,7 +21412,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="41c9fafd-c058-44f8-b2ce-53cd3afba157" xsi:nil="true"/>
@@ -18000,15 +21423,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4A9A146-E1D4-411F-BBA2-056A85056DA8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{118099E9-5674-4C43-BF01-17622689F55A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18027,7 +21451,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F24CF1C-E15F-4170-99B6-AB935727F795}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -18036,4 +21460,12 @@
     <ds:schemaRef ds:uri="3c9f7625-f508-4699-980b-15a788d55c32"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4A9A146-E1D4-411F-BBA2-056A85056DA8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>